<commit_message>
initial commit: revisi data keluhan
</commit_message>
<xml_diff>
--- a/keluhan baru.xlsx
+++ b/keluhan baru.xlsx
@@ -5,22 +5,22 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adity\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\magang smt 6\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79EABC17-C2F2-45E3-BF32-2D5AD70B2DC3}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{753CA9ED-86B3-4B0F-8929-482052740DA5}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="15200" windowHeight="7520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="191029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3007" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3067" uniqueCount="99">
   <si>
     <t>CUSTOMER_ID</t>
   </si>
@@ -261,12 +261,69 @@
   <si>
     <t>High Tarif</t>
   </si>
+  <si>
+    <t>janji temu perbaikan instalasi selalu diundur tanpa kejelasan sudah terjadi beberapa hari</t>
+  </si>
+  <si>
+    <t>tagihan pju di wilayah kami naik drastis</t>
+  </si>
+  <si>
+    <t>lonjakan biaya listrik tidak wajar dari bulan sebelumnya tolong dibantu</t>
+  </si>
+  <si>
+    <t>meteran sering anjlok padahal pemakaian elektronik normal</t>
+  </si>
+  <si>
+    <t>token yang dibeli selalu gagal dimasukkan muncul tulisan reject mohon segera ditindaklanjuti</t>
+  </si>
+  <si>
+    <t>meteran sering anjlok padahal pemakaian elektronik normal mohon segera ditindaklanjuti</t>
+  </si>
+  <si>
+    <t>aplikasi sering force close saat mau buat laporan gangguan tolong dibantu</t>
+  </si>
+  <si>
+    <t>token yang dibeli selalu gagal dimasukkan muncul tulisan reject</t>
+  </si>
+  <si>
+    <t>permohonan pemindahan tiang listrik di depan pagar rumah tolong dibantu</t>
+  </si>
+  <si>
+    <t>lonjakan biaya listrik tidak wajar dari bulan sebelumnya</t>
+  </si>
+  <si>
+    <t>alarm token berbunyi terus padahal kuota masih banyak mohon segera ditindaklanjuti</t>
+  </si>
+  <si>
+    <t>permohonan pemindahan tiang listrik di depan pagar rumah mohon segera ditindaklanjuti</t>
+  </si>
+  <si>
+    <t>mohon relokasi kabel instalasi yang melorot ke jalan sudah terjadi beberapa hari</t>
+  </si>
+  <si>
+    <t>alarm token berbunyi terus padahal kuota masih banyak</t>
+  </si>
+  <si>
+    <t>tiang listrik miring setelah ditabrak kendaraan mohon segera ditindaklanjuti</t>
+  </si>
+  <si>
+    <t>angka stan meter di lapangan berbeda jauh dengan tagihan mohon segera ditindaklanjuti</t>
+  </si>
+  <si>
+    <t>respon pengaduan di aplikasi terkesan lambat dan monoton sudah terjadi beberapa hari</t>
+  </si>
+  <si>
+    <t>call center sulit dihubungi selalu sibuk sudah terjadi beberapa hari</t>
+  </si>
+  <si>
+    <t>tagihan bulan ini membengkak padahal rumah kosong mohon segera ditindaklanjuti</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -282,6 +339,12 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -291,7 +354,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -314,14 +377,38 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -661,8 +748,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G1001"/>
+  <dimension ref="A1:G1021"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="6" max="6" width="8.90625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
@@ -23664,7 +23754,7 @@
         <v>555</v>
       </c>
     </row>
-    <row r="1001" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="1001" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1001">
         <v>999</v>
       </c>
@@ -23687,7 +23777,487 @@
         <v>110</v>
       </c>
     </row>
+    <row r="1002" spans="1:7" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A1002">
+        <v>1000</v>
+      </c>
+      <c r="B1002" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="C1002" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="D1002" s="4">
+        <v>51808</v>
+      </c>
+      <c r="E1002" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1002" s="2">
+        <v>183272</v>
+      </c>
+      <c r="G1002" s="4">
+        <v>866</v>
+      </c>
+    </row>
+    <row r="1003" spans="1:7" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A1003">
+        <f>A1002+1</f>
+        <v>1001</v>
+      </c>
+      <c r="B1003" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="C1003" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="D1003" s="4">
+        <v>51808</v>
+      </c>
+      <c r="E1003" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="F1003" s="2">
+        <v>215421</v>
+      </c>
+      <c r="G1003" s="4">
+        <v>509</v>
+      </c>
+    </row>
+    <row r="1004" spans="1:7" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A1004">
+        <f t="shared" ref="A1004:A1021" si="0">A1003+1</f>
+        <v>1002</v>
+      </c>
+      <c r="B1004" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="C1004" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="D1004" s="4">
+        <v>51808</v>
+      </c>
+      <c r="E1004" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1004" s="2">
+        <v>688353</v>
+      </c>
+      <c r="G1004" s="4">
+        <v>995</v>
+      </c>
+    </row>
+    <row r="1005" spans="1:7" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A1005">
+        <f t="shared" si="0"/>
+        <v>1003</v>
+      </c>
+      <c r="B1005" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="C1005" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="D1005" s="4">
+        <v>51808</v>
+      </c>
+      <c r="E1005" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="F1005" s="2">
+        <v>418501</v>
+      </c>
+      <c r="G1005" s="4">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="1006" spans="1:7" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A1006">
+        <f t="shared" si="0"/>
+        <v>1004</v>
+      </c>
+      <c r="B1006" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="C1006" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="D1006" s="4">
+        <v>51808</v>
+      </c>
+      <c r="E1006" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="F1006" s="2">
+        <v>82265</v>
+      </c>
+      <c r="G1006" s="4">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="1007" spans="1:7" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A1007">
+        <f t="shared" si="0"/>
+        <v>1005</v>
+      </c>
+      <c r="B1007" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="C1007" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="D1007" s="4">
+        <v>51808</v>
+      </c>
+      <c r="E1007" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1007" s="2">
+        <v>498982</v>
+      </c>
+      <c r="G1007" s="4">
+        <v>701</v>
+      </c>
+    </row>
+    <row r="1008" spans="1:7" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A1008">
+        <f t="shared" si="0"/>
+        <v>1006</v>
+      </c>
+      <c r="B1008" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="C1008" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="D1008" s="4">
+        <v>51808</v>
+      </c>
+      <c r="E1008" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="F1008" s="2">
+        <v>139613</v>
+      </c>
+      <c r="G1008" s="4">
+        <v>776</v>
+      </c>
+    </row>
+    <row r="1009" spans="1:7" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A1009">
+        <f t="shared" si="0"/>
+        <v>1007</v>
+      </c>
+      <c r="B1009" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="C1009" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="D1009" s="4">
+        <v>51808</v>
+      </c>
+      <c r="E1009" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="F1009" s="2">
+        <v>184633</v>
+      </c>
+      <c r="G1009" s="4">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="1010" spans="1:7" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A1010">
+        <f t="shared" si="0"/>
+        <v>1008</v>
+      </c>
+      <c r="B1010" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="C1010" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="D1010" s="4">
+        <v>51808</v>
+      </c>
+      <c r="E1010" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="F1010" s="2">
+        <v>168259</v>
+      </c>
+      <c r="G1010" s="4">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="1011" spans="1:7" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A1011">
+        <f t="shared" si="0"/>
+        <v>1009</v>
+      </c>
+      <c r="B1011" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="C1011" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="D1011" s="4">
+        <v>51808</v>
+      </c>
+      <c r="E1011" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="F1011" s="2">
+        <v>481413</v>
+      </c>
+      <c r="G1011" s="4">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="1012" spans="1:7" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A1012">
+        <f t="shared" si="0"/>
+        <v>1010</v>
+      </c>
+      <c r="B1012" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="C1012" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="D1012" s="4">
+        <v>51808</v>
+      </c>
+      <c r="E1012" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="F1012" s="2">
+        <v>311233</v>
+      </c>
+      <c r="G1012" s="4">
+        <v>647</v>
+      </c>
+    </row>
+    <row r="1013" spans="1:7" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A1013">
+        <f t="shared" si="0"/>
+        <v>1011</v>
+      </c>
+      <c r="B1013" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="C1013" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="D1013" s="4">
+        <v>51808</v>
+      </c>
+      <c r="E1013" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="F1013" s="2">
+        <v>309178</v>
+      </c>
+      <c r="G1013" s="4">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="1014" spans="1:7" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A1014">
+        <f t="shared" si="0"/>
+        <v>1012</v>
+      </c>
+      <c r="B1014" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="C1014" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="D1014" s="4">
+        <v>51808</v>
+      </c>
+      <c r="E1014" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="F1014" s="2">
+        <v>623167</v>
+      </c>
+      <c r="G1014" s="4">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="1015" spans="1:7" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A1015">
+        <f t="shared" si="0"/>
+        <v>1013</v>
+      </c>
+      <c r="B1015" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="C1015" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="D1015" s="4">
+        <v>51808</v>
+      </c>
+      <c r="E1015" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="F1015" s="2">
+        <v>344972</v>
+      </c>
+      <c r="G1015" s="4">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="1016" spans="1:7" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A1016">
+        <f t="shared" si="0"/>
+        <v>1014</v>
+      </c>
+      <c r="B1016" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="C1016" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="D1016" s="4">
+        <v>51808</v>
+      </c>
+      <c r="E1016" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="F1016" s="2">
+        <v>145419</v>
+      </c>
+      <c r="G1016" s="4">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="1017" spans="1:7" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A1017">
+        <f t="shared" si="0"/>
+        <v>1015</v>
+      </c>
+      <c r="B1017" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="C1017" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="D1017" s="4">
+        <v>51808</v>
+      </c>
+      <c r="E1017" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="F1017" s="2">
+        <v>114774</v>
+      </c>
+      <c r="G1017" s="4">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="1018" spans="1:7" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A1018">
+        <f t="shared" si="0"/>
+        <v>1016</v>
+      </c>
+      <c r="B1018" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="C1018" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="D1018" s="4">
+        <v>51808</v>
+      </c>
+      <c r="E1018" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1018" s="2">
+        <v>307726</v>
+      </c>
+      <c r="G1018" s="4">
+        <v>557</v>
+      </c>
+    </row>
+    <row r="1019" spans="1:7" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A1019">
+        <f t="shared" si="0"/>
+        <v>1017</v>
+      </c>
+      <c r="B1019" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="C1019" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="D1019" s="4">
+        <v>51808</v>
+      </c>
+      <c r="E1019" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1019" s="2">
+        <v>300957</v>
+      </c>
+      <c r="G1019" s="4">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="1020" spans="1:7" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A1020">
+        <f t="shared" si="0"/>
+        <v>1018</v>
+      </c>
+      <c r="B1020" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="C1020" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="D1020" s="4">
+        <v>51808</v>
+      </c>
+      <c r="E1020" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="F1020" s="2">
+        <v>288756</v>
+      </c>
+      <c r="G1020" s="4">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="1021" spans="1:7" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A1021">
+        <f t="shared" si="0"/>
+        <v>1019</v>
+      </c>
+      <c r="B1021" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="C1021" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="D1021" s="4">
+        <v>51808</v>
+      </c>
+      <c r="E1021" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1021" s="2">
+        <v>200701</v>
+      </c>
+      <c r="G1021" s="4">
+        <v>58</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>